<commit_message>
Contribution analysis ok and SI organization
</commit_message>
<xml_diff>
--- a/data/Mappings/MAPPINGS_EI.xlsx
+++ b/data/Mappings/MAPPINGS_EI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/regionalized_lci_mineral/data/Mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="571" documentId="13_ncr:1_{7529039C-DAB5-4502-A4FA-B91C5ABC1E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{729C53C0-516D-43AF-8E24-5952EA0ADB4C}"/>
+  <xr:revisionPtr revIDLastSave="575" documentId="13_ncr:1_{7529039C-DAB5-4502-A4FA-B91C5ABC1E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9C8CDF1-F64D-45C0-8CE9-FB645F3FAC33}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2238,7 +2238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2270,7 +2270,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17635,6 +17634,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B7552F2-809E-47BC-A2F4-BF83969FDA26}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -17678,7 +17678,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>425</v>
       </c>
@@ -17704,7 +17704,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>425</v>
       </c>
@@ -17730,7 +17730,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>425</v>
       </c>
@@ -17759,7 +17759,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>425</v>
       </c>
@@ -17785,7 +17785,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>425</v>
       </c>
@@ -17814,7 +17814,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>424</v>
       </c>
@@ -17843,7 +17843,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>425</v>
       </c>
@@ -17869,7 +17869,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>425</v>
       </c>
@@ -17898,7 +17898,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>425</v>
       </c>
@@ -18043,7 +18043,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>425</v>
       </c>
@@ -18095,7 +18095,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>424</v>
       </c>
@@ -18121,7 +18121,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>424</v>
       </c>
@@ -18147,7 +18147,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>424</v>
       </c>
@@ -18173,7 +18173,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>424</v>
       </c>
@@ -18199,7 +18199,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>424</v>
       </c>
@@ -18225,7 +18225,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>424</v>
       </c>
@@ -18254,7 +18254,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>424</v>
       </c>
@@ -18283,7 +18283,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>424</v>
       </c>
@@ -18312,7 +18312,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>424</v>
       </c>
@@ -18341,7 +18341,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>424</v>
       </c>
@@ -18367,7 +18367,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>425</v>
       </c>
@@ -18396,7 +18396,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>424</v>
       </c>
@@ -18425,7 +18425,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>425</v>
       </c>
@@ -18454,7 +18454,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>424</v>
       </c>
@@ -18480,7 +18480,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>424</v>
       </c>
@@ -18506,7 +18506,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>424</v>
       </c>
@@ -18532,7 +18532,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>424</v>
       </c>
@@ -18558,7 +18558,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>424</v>
       </c>
@@ -18584,7 +18584,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>424</v>
       </c>
@@ -18610,7 +18610,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>424</v>
       </c>
@@ -18636,7 +18636,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>425</v>
       </c>
@@ -18665,7 +18665,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>425</v>
       </c>
@@ -18691,7 +18691,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>425</v>
       </c>
@@ -18720,7 +18720,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>425</v>
       </c>
@@ -18749,7 +18749,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>425</v>
       </c>
@@ -18778,7 +18778,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>425</v>
       </c>
@@ -18807,7 +18807,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>425</v>
       </c>
@@ -18836,7 +18836,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>425</v>
       </c>
@@ -18865,7 +18865,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>424</v>
       </c>
@@ -18894,7 +18894,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>425</v>
       </c>
@@ -18923,7 +18923,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>425</v>
       </c>
@@ -18952,7 +18952,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>425</v>
       </c>
@@ -18978,7 +18978,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>424</v>
       </c>
@@ -19004,11 +19004,11 @@
         <v>175</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>424</v>
       </c>
-      <c r="B50" s="25" t="s">
+      <c r="B50" t="s">
         <v>1</v>
       </c>
       <c r="C50" s="6" t="s">
@@ -19030,7 +19030,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>424</v>
       </c>
@@ -19056,7 +19056,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>425</v>
       </c>
@@ -19085,7 +19085,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>424</v>
       </c>
@@ -19111,7 +19111,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>424</v>
       </c>
@@ -19137,7 +19137,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>425</v>
       </c>
@@ -19163,7 +19163,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>425</v>
       </c>
@@ -19189,7 +19189,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>425</v>
       </c>
@@ -19215,7 +19215,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>424</v>
       </c>
@@ -19241,7 +19241,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>424</v>
       </c>
@@ -19267,7 +19267,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>424</v>
       </c>
@@ -19293,7 +19293,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>424</v>
       </c>
@@ -19319,7 +19319,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>425</v>
       </c>
@@ -19348,7 +19348,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>425</v>
       </c>
@@ -19377,7 +19377,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>425</v>
       </c>
@@ -19403,7 +19403,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>425</v>
       </c>
@@ -19429,7 +19429,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>425</v>
       </c>
@@ -19455,7 +19455,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>425</v>
       </c>
@@ -19481,7 +19481,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>425</v>
       </c>
@@ -19507,7 +19507,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>424</v>
       </c>
@@ -19533,7 +19533,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>424</v>
       </c>
@@ -19559,7 +19559,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>424</v>
       </c>
@@ -19585,7 +19585,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>424</v>
       </c>
@@ -19611,7 +19611,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>425</v>
       </c>
@@ -19640,7 +19640,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>425</v>
       </c>
@@ -19666,7 +19666,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>425</v>
       </c>
@@ -19692,7 +19692,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>424</v>
       </c>
@@ -19718,7 +19718,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>425</v>
       </c>
@@ -19747,7 +19747,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>424</v>
       </c>
@@ -19773,7 +19773,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>425</v>
       </c>
@@ -19802,7 +19802,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>425</v>
       </c>
@@ -19828,7 +19828,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>425</v>
       </c>
@@ -19857,7 +19857,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>425</v>
       </c>
@@ -19886,7 +19886,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>425</v>
       </c>
@@ -19915,7 +19915,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>425</v>
       </c>
@@ -19941,7 +19941,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>425</v>
       </c>
@@ -19967,7 +19967,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>425</v>
       </c>
@@ -19996,7 +19996,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>425</v>
       </c>
@@ -20025,7 +20025,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>425</v>
       </c>
@@ -20054,7 +20054,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>425</v>
       </c>
@@ -20083,7 +20083,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>425</v>
       </c>
@@ -20112,7 +20112,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>425</v>
       </c>
@@ -20138,7 +20138,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>425</v>
       </c>
@@ -20164,11 +20164,11 @@
         <v>175</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>425</v>
       </c>
-      <c r="B93" s="25" t="s">
+      <c r="B93" t="s">
         <v>55</v>
       </c>
       <c r="C93" s="6" t="s">
@@ -20193,11 +20193,11 @@
         <v>221</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>425</v>
       </c>
-      <c r="B94" s="25" t="s">
+      <c r="B94" t="s">
         <v>515</v>
       </c>
       <c r="C94" s="6" t="s">
@@ -20220,7 +20220,7 @@
       </c>
       <c r="I94" s="17"/>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>425</v>
       </c>
@@ -20247,7 +20247,7 @@
       </c>
       <c r="I95" s="17"/>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>425</v>
       </c>
@@ -20274,11 +20274,11 @@
       </c>
       <c r="I96" s="17"/>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>425</v>
       </c>
-      <c r="B97" s="25" t="s">
+      <c r="B97" t="s">
         <v>43</v>
       </c>
       <c r="C97" s="6" t="s">
@@ -20303,11 +20303,11 @@
         <v>209</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>425</v>
       </c>
-      <c r="B98" s="25" t="s">
+      <c r="B98" t="s">
         <v>420</v>
       </c>
       <c r="C98" s="6" t="s">
@@ -20329,11 +20329,11 @@
         <v>175</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>425</v>
       </c>
-      <c r="B99" s="25" t="s">
+      <c r="B99" t="s">
         <v>63</v>
       </c>
       <c r="C99" s="6" t="s">
@@ -20355,7 +20355,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>425</v>
       </c>
@@ -20381,7 +20381,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>425</v>
       </c>
@@ -20410,6 +20410,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I101" xr:uid="{2B7552F2-809E-47BC-A2F4-BF83969FDA26}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Collectors"/>
+        <filter val="Collectors (xanthates)"/>
+        <filter val="Copper sulfate"/>
+        <filter val="Frother"/>
+        <filter val="Frother (MIBC or Dowfroth)"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I101">
       <sortCondition ref="F1:F101"/>
     </sortState>

</xml_diff>